<commit_message>
Backend completed- csv and authentication
</commit_message>
<xml_diff>
--- a/SmartIMS_Development_Timeline.xlsx
+++ b/SmartIMS_Development_Timeline.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\swapn\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Darshana\Desktop\Maxxzoom_task\Inventora\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B24CE42-3E00-40B1-BC41-379232BA5C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9252"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -249,7 +250,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -313,13 +314,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -339,9 +343,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -379,9 +383,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -416,7 +420,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -451,7 +455,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -624,17 +628,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" customWidth="1"/>
-    <col min="4" max="4" width="121.109375" customWidth="1"/>
-    <col min="5" max="5" width="23.6640625" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="36.28515625" customWidth="1"/>
+    <col min="4" max="4" width="121.140625" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -651,7 +655,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -665,7 +669,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -679,7 +683,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -693,7 +697,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -707,7 +711,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -721,7 +725,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -735,7 +739,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -749,7 +753,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -763,7 +767,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -777,7 +781,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -791,7 +795,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -805,7 +809,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -819,7 +823,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -829,11 +833,11 @@
       <c r="C14" t="s">
         <v>46</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -847,7 +851,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>

</xml_diff>